<commit_message>
Parameters, big meeting, all that
</commit_message>
<xml_diff>
--- a/Assignment 9/Parameters_copy.xlsx
+++ b/Assignment 9/Parameters_copy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29819"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29825"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://purdue0-my.sharepoint.com/personal/hong411_purdue_edu/Documents/AAE 451/Assignment 8/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{23B97E16-C638-4182-AF0F-0CC473A14F45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D41534BB-ED0C-4A84-BD08-3AB77DF42207}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15820" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15820" firstSheet="12" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Deliverables and tasks" sheetId="2" r:id="rId1"/>
@@ -264,7 +264,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="869" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="869" uniqueCount="185">
   <si>
     <t>Deliverables</t>
   </si>
@@ -725,7 +725,13 @@
     <t>no nacelles no fuselage</t>
   </si>
   <si>
+    <t>These three are in radians!</t>
+  </si>
+  <si>
     <t>idk man, set to 0</t>
+  </si>
+  <si>
+    <t>idk man, set to 0.9</t>
   </si>
   <si>
     <t>things to chekc</t>
@@ -933,7 +939,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -964,6 +970,12 @@
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -977,7 +989,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -994,6 +1006,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -24284,7 +24297,7 @@
     <row r="16" spans="2:21">
       <c r="D16">
         <f>(D5*D6)/(D23*D24)</f>
-        <v>5.0671797001708048E-3</v>
+        <v>4.5296154234682872E-3</v>
       </c>
       <c r="L16" t="s">
         <v>35</v>
@@ -24302,7 +24315,7 @@
       </c>
       <c r="I17">
         <f>(I5*I6)/(D24*D25)</f>
-        <v>1.5239222026882683E-3</v>
+        <v>1.580951432545925E-3</v>
       </c>
     </row>
     <row r="20" spans="2:9">
@@ -24340,7 +24353,7 @@
       </c>
       <c r="D23">
         <f>Sunfish!B2*0.5*3.28084</f>
-        <v>18.044619999999998</v>
+        <v>19.685040000000001</v>
       </c>
       <c r="G23" t="s">
         <v>147</v>
@@ -24352,7 +24365,7 @@
       </c>
       <c r="D24">
         <f>0.5*D25*3.28084*Sunfish!B2</f>
-        <v>1082.6772000000001</v>
+        <v>1110.2362560000001</v>
       </c>
       <c r="G24" t="s">
         <v>148</v>
@@ -24363,7 +24376,7 @@
         <v>40</v>
       </c>
       <c r="D25">
-        <v>60</v>
+        <v>56.4</v>
       </c>
       <c r="G25" t="s">
         <v>149</v>
@@ -24375,7 +24388,7 @@
       </c>
       <c r="D26">
         <f>D25^2/D24</f>
-        <v>3.3250908026880031</v>
+        <v>2.8651199083161627</v>
       </c>
       <c r="G26" t="s">
         <v>51</v>
@@ -24581,27 +24594,22 @@
     </row>
     <row r="2" spans="1:45">
       <c r="A2">
-        <f>'Sizing - Sunfish_final'!D23 * 0.3048</f>
-        <v>5.5000001759999995</v>
+        <v>5.5</v>
       </c>
       <c r="B2">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2">
-        <f>('Sizing - Sunfish_final'!D8 + 'Sizing - Sunfish_final'!D9)* 0.3048 / 2</f>
-        <v>0.76200000000000001</v>
+        <v>2.4900000000000002</v>
       </c>
       <c r="D2">
-        <f>('Sizing - Sunfish_final'!I8 + 'Sizing - Sunfish_final'!I9)* 0.3048 / 2</f>
-        <v>0.76200000000000001</v>
+        <v>2.4900000000000002</v>
       </c>
       <c r="E2">
-        <f>'Sizing - Sunfish_final'!D25 * 0.3048</f>
-        <v>18.288</v>
+        <v>17.2</v>
       </c>
       <c r="F2">
-        <f>'Sizing - Sunfish_final'!D6</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -24616,8 +24624,7 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <f>'Sizing - Sunfish_final'!D24 * 0.09290304</f>
-        <v>100.58400321868801</v>
+        <v>111.8</v>
       </c>
       <c r="L2">
         <f>'Sizing - Sunfish_final'!D5</f>
@@ -24628,12 +24635,12 @@
         <v>12.374368675682753</v>
       </c>
       <c r="N2">
-        <f>'Sizing - Sunfish_final'!D24 * 0.09290304</f>
-        <v>100.58400321868801</v>
+        <f>K2</f>
+        <v>111.8</v>
       </c>
       <c r="O2">
-        <f>('Sizing - Sunfish_final'!D27) * PI() / 180</f>
-        <v>0.58992128717408332</v>
+        <f>RADIANS(38)</f>
+        <v>0.66322511575784526</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -24643,7 +24650,7 @@
       </c>
       <c r="R2">
         <f>'Sizing - Sunfish_final'!D26</f>
-        <v>3.3250908026880031</v>
+        <v>2.8651199083161627</v>
       </c>
       <c r="S2">
         <f>'Sizing - Sunfish_final'!I11</f>
@@ -24658,7 +24665,7 @@
       </c>
       <c r="V2">
         <f>B2*0.25</f>
-        <v>2.75</v>
+        <v>3</v>
       </c>
       <c r="W2">
         <v>0.9</v>
@@ -24696,7 +24703,7 @@
       </c>
       <c r="AH2">
         <f>F2</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AI2" s="11"/>
     </row>
@@ -24820,13 +24827,13 @@
         <v>152</v>
       </c>
       <c r="O5" t="s">
-        <v>97</v>
+        <v>153</v>
       </c>
       <c r="U5" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="W5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="6" spans="1:45">
@@ -24836,53 +24843,53 @@
     </row>
     <row r="7" spans="1:45">
       <c r="A7" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="V7" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="1:45">
       <c r="A8" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" spans="1:45">
       <c r="A9" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" spans="1:45">
       <c r="A10" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11" spans="1:45">
       <c r="A11" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="12" spans="1:45">
       <c r="A12" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13" spans="1:45">
       <c r="A13" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="14" spans="1:45">
       <c r="A14" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15" spans="1:45">
       <c r="A15" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C15" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -25220,7 +25227,7 @@
         <v>109</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>112</v>
@@ -25235,10 +25242,10 @@
         <v>120</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H1" s="13" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="I1" s="13" t="s">
         <v>110</v>
@@ -25272,8 +25279,8 @@
       <c r="C2" s="11">
         <v>-2.5000000000000001E-2</v>
       </c>
-      <c r="D2" s="11">
-        <v>1.3</v>
+      <c r="D2" s="16">
+        <v>1.5</v>
       </c>
       <c r="E2" s="11">
         <v>0.9</v>
@@ -25359,7 +25366,7 @@
     <row r="5" spans="1:15">
       <c r="C5" s="9"/>
       <c r="L5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -25367,32 +25374,32 @@
     </row>
     <row r="16" spans="1:15">
       <c r="C16" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="17" spans="3:3">
       <c r="C17" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="18" spans="3:3">
       <c r="C18" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="19" spans="3:3">
       <c r="C19" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="20" spans="3:3">
       <c r="C20" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="21" spans="3:3">
       <c r="C21" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -25413,7 +25420,7 @@
         <v>109</v>
       </c>
       <c r="B1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C1" t="s">
         <v>112</v>
@@ -25428,10 +25435,10 @@
         <v>120</v>
       </c>
       <c r="G1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="I1" t="s">
         <v>110</v>
@@ -25554,12 +25561,12 @@
     <row r="5" spans="1:15">
       <c r="C5" s="9"/>
       <c r="L5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6" spans="1:15">
       <c r="L6" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -25567,32 +25574,32 @@
     </row>
     <row r="16" spans="1:15">
       <c r="C16" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="17" spans="3:3">
       <c r="C17" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="18" spans="3:3">
       <c r="C18" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="19" spans="3:3">
       <c r="C19" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="20" spans="3:3">
       <c r="C20" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="21" spans="3:3">
       <c r="C21" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -25610,7 +25617,7 @@
         <v>109</v>
       </c>
       <c r="B1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C1" t="s">
         <v>112</v>
@@ -25625,10 +25632,10 @@
         <v>120</v>
       </c>
       <c r="G1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="I1" t="s">
         <v>110</v>
@@ -25699,10 +25706,10 @@
         <v>12</v>
       </c>
       <c r="Q2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="R2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -25752,10 +25759,10 @@
         <v>13.5</v>
       </c>
       <c r="Q3" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="R3" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -25811,45 +25818,45 @@
     <row r="7" spans="1:18">
       <c r="C7" s="9"/>
       <c r="H7" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="O7" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="8" spans="1:18">
       <c r="F8" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="16" spans="1:18">
       <c r="C16" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="17" spans="3:3">
       <c r="C17" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="18" spans="3:3">
       <c r="C18" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="19" spans="3:3">
       <c r="C19" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="20" spans="3:3">
       <c r="C20" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="21" spans="3:3">
       <c r="C21" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>